<commit_message>
docs: actualizar Fase 2 con evidencias grupales, individuales y de proyecto completas
</commit_message>
<xml_diff>
--- a/Fase 2/Evidencias Grupales/MATRIZ DE RIESGO.xlsx
+++ b/Fase 2/Evidencias Grupales/MATRIZ DE RIESGO.xlsx
@@ -1,132 +1,118 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27726"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jeanette Leonelli\Desktop\2024-1\PTY4478\Fase2\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66C638A2-FD8E-4F78-9DE8-8BFBE2EF976B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="MATRIZ" sheetId="1" r:id="rId1"/>
-    <sheet name="DICCIONARIO" sheetId="2" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MATRIZ" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DICCIONARIO" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="22">
-  <si>
-    <t>Riesgo</t>
-  </si>
-  <si>
-    <t>Categoría</t>
-  </si>
-  <si>
-    <t>Probabilidad</t>
-  </si>
-  <si>
-    <t>Impacto</t>
-  </si>
-  <si>
-    <t>Acción de Mitigación</t>
-  </si>
-  <si>
-    <t>Responsable</t>
-  </si>
-  <si>
-    <t>Desarrollo</t>
-  </si>
-  <si>
-    <t>Proyecto</t>
-  </si>
-  <si>
-    <t>Despreciable: Poco relevante.</t>
-  </si>
-  <si>
-    <t>Marginal: Su impacto debe ser tenido en cuenta, pero no afecta factores claves del proyecto.</t>
-  </si>
-  <si>
-    <t>Crítica: Podría afectar de manera sustancial al proyecto y podría impedir su conclusión/término de manera exitosa.</t>
-  </si>
-  <si>
-    <t>Catastrófica: Significaría el fracaso del proyecto o afectaría gravemente la ejecución/continuación/termino del mismo</t>
-  </si>
-  <si>
-    <t>IMPACTO</t>
-  </si>
-  <si>
-    <t>ID</t>
-  </si>
-  <si>
-    <t>Muy Bajo (Menos del 10%)</t>
-  </si>
-  <si>
-    <t>Medio (Entre  41 % y 80%)</t>
-  </si>
-  <si>
-    <t>Alto (Mas del 81%)</t>
-  </si>
-  <si>
-    <t>Bajo (Entre del 11% y 40%)</t>
-  </si>
-  <si>
-    <t>Categoria</t>
-  </si>
-  <si>
-    <t>Externo</t>
-  </si>
-  <si>
-    <t>Naturaleza</t>
-  </si>
-  <si>
-    <t>ID RIESGO</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="16">
     <font>
+      <name val="Arial"/>
+      <color rgb="FF000000"/>
       <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
+      <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="12"/>
-      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="10"/>
     </font>
     <font>
-      <sz val="10"/>
       <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="12"/>
     </font>
     <font>
-      <b/>
+      <name val="Arial"/>
+      <color rgb="FF000000"/>
       <sz val="10"/>
-      <name val="Arial"/>
     </font>
     <font>
-      <b/>
+      <name val="Arial"/>
+      <color theme="1"/>
       <sz val="10"/>
-      <name val="Arial"/>
     </font>
     <font>
+      <name val="Noto Sans Symbols"/>
+      <color theme="1"/>
       <sz val="10"/>
-      <name val="Noto Sans Symbols"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <color theme="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <sz val="8"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="15"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="009C5700"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00006100"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="007F6000"/>
+      <sz val="9"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="15">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -139,30 +125,78 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CB"/>
+        <bgColor rgb="FFFFF2CB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFDBE5F1"/>
         <bgColor rgb="FFDBE5F1"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
+        <fgColor rgb="FFC5E0B3"/>
+        <bgColor rgb="FFC5E0B3"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
+        <fgColor rgb="FFF4B083"/>
+        <bgColor rgb="FFF4B083"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.39997558519241921"/>
-        <bgColor indexed="64"/>
+        <fgColor rgb="001F4E79"/>
+        <bgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6E4F0"/>
+        <bgColor rgb="00D6E4F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E75B6"/>
+        <bgColor rgb="002E75B6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F7FA"/>
+        <bgColor rgb="00F2F7FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+        <bgColor rgb="00FFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+        <bgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+        <bgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -196,91 +230,225 @@
       </bottom>
       <diagonal/>
     </border>
+    <border/>
     <border>
       <left style="thin">
-        <color indexed="64"/>
+        <color rgb="00FFFFFF"/>
       </left>
       <right style="thin">
-        <color indexed="64"/>
+        <color rgb="00FFFFFF"/>
       </right>
       <top style="thin">
-        <color indexed="64"/>
+        <color rgb="001F4E79"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="001F4E79"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
       </top>
       <bottom style="thin">
-        <color indexed="64"/>
+        <color rgb="00D9D9D9"/>
       </bottom>
-      <diagonal/>
+    </border>
+    <border>
+      <top style="medium">
+        <color rgb="002E75B6"/>
+      </top>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+  <cellXfs count="39">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="11" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="13" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="14" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Sheets">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
+        <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546A"/>
+        <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E7E6E6"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt2>
       <a:accent1>
         <a:srgbClr val="4472C4"/>
@@ -304,116 +472,22 @@
         <a:srgbClr val="0563C1"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954F72"/>
+        <a:srgbClr val="0563C1"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Sheets">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック Light"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线 Light"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
+        <a:latin typeface="Arial"/>
+        <a:ea typeface="Arial"/>
+        <a:cs typeface="Arial"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
+        <a:latin typeface="Arial"/>
+        <a:ea typeface="Arial"/>
+        <a:cs typeface="Arial"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -553,249 +627,1174 @@
   </a:themeElements>
   <a:objectDefaults/>
   <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1005"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="14.3984375" defaultRowHeight="15" customHeight="1"/>
+  <dimension ref="A1:N39"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="2" max="2" width="33" customWidth="1"/>
-    <col min="3" max="5" width="14.3984375" customWidth="1"/>
-    <col min="6" max="6" width="66.86328125" customWidth="1"/>
-    <col min="7" max="7" width="23.86328125" customWidth="1"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="13" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="13" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="14" bestFit="1" customWidth="1" min="5" max="5"/>
+    <col width="15" bestFit="1" customWidth="1" min="6" max="6"/>
+    <col width="46" customWidth="1" min="7" max="7"/>
+    <col width="42" customWidth="1" min="8" max="26"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15.75" customHeight="1">
-      <c r="A1" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" ht="15.75" customHeight="1">
-      <c r="A2" s="2"/>
-      <c r="B2" s="2"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-    </row>
-    <row r="3" spans="1:7" ht="15.75" customHeight="1">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4"/>
-    </row>
-    <row r="4" spans="1:7" ht="15.75" customHeight="1">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
-    </row>
-    <row r="5" spans="1:7" ht="15.75" customHeight="1">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
-    </row>
-    <row r="6" spans="1:7" ht="15.75" customHeight="1">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="4"/>
-      <c r="G6" s="4"/>
-    </row>
-    <row r="7" spans="1:7" ht="15.75" customHeight="1">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="4"/>
-      <c r="G7" s="4"/>
-    </row>
-    <row r="8" spans="1:7" ht="15.75" customHeight="1">
-      <c r="A8" s="2"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
-      <c r="F8" s="4"/>
-      <c r="G8" s="4"/>
-    </row>
-    <row r="9" spans="1:7" ht="15.75" customHeight="1">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="4"/>
-      <c r="G9" s="4"/>
-    </row>
-    <row r="10" spans="1:7" ht="15.75" customHeight="1">
-      <c r="A10" s="2"/>
-      <c r="B10" s="2"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
-      <c r="F10" s="4"/>
-      <c r="G10" s="4"/>
-    </row>
-    <row r="11" spans="1:7" ht="15.75" customHeight="1">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-      <c r="F11" s="4"/>
-      <c r="G11" s="4"/>
-    </row>
-    <row r="12" spans="1:7" ht="15.75" customHeight="1">
-      <c r="A12" s="2"/>
-      <c r="B12" s="2"/>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3"/>
-      <c r="F12" s="4"/>
-      <c r="G12" s="4"/>
-    </row>
-    <row r="13" spans="1:7" ht="15.75" customHeight="1">
-      <c r="A13" s="2"/>
-      <c r="B13" s="2"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
-      <c r="F13" s="4"/>
-      <c r="G13" s="4"/>
-    </row>
-    <row r="14" spans="1:7" ht="15.75" customHeight="1">
-      <c r="A14" s="2"/>
-      <c r="B14" s="2"/>
-      <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
-      <c r="F14" s="4"/>
-      <c r="G14" s="4"/>
-    </row>
-    <row r="15" spans="1:7" ht="15.75" customHeight="1">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
-      <c r="E15" s="3"/>
-      <c r="F15" s="4"/>
-      <c r="G15" s="4"/>
-    </row>
-    <row r="16" spans="1:7" ht="15.75" customHeight="1">
-      <c r="A16" s="2"/>
-      <c r="B16" s="2"/>
-      <c r="C16" s="3"/>
-      <c r="D16" s="3"/>
-      <c r="E16" s="3"/>
-      <c r="F16" s="4"/>
-      <c r="G16" s="4"/>
-    </row>
-    <row r="17" spans="1:7" ht="15.75" customHeight="1">
-      <c r="A17" s="2"/>
-      <c r="B17" s="2"/>
-      <c r="C17" s="3"/>
-      <c r="D17" s="3"/>
-      <c r="E17" s="3"/>
-      <c r="F17" s="4"/>
-      <c r="G17" s="4"/>
-    </row>
-    <row r="18" spans="1:7" ht="15.75" customHeight="1">
-      <c r="A18" s="2"/>
-      <c r="B18" s="2"/>
-      <c r="C18" s="3"/>
-      <c r="D18" s="3"/>
-      <c r="E18" s="3"/>
-      <c r="F18" s="4"/>
-      <c r="G18" s="4"/>
-    </row>
-    <row r="19" spans="1:7" ht="15.75" customHeight="1">
-      <c r="A19" s="2"/>
-      <c r="B19" s="2"/>
-      <c r="C19" s="3"/>
-      <c r="D19" s="3"/>
-      <c r="E19" s="3"/>
-      <c r="F19" s="4"/>
-      <c r="G19" s="4"/>
-    </row>
-    <row r="20" spans="1:7" ht="15.75" customHeight="1">
-      <c r="A20" s="2"/>
-      <c r="B20" s="2"/>
-      <c r="C20" s="3"/>
-      <c r="D20" s="3"/>
-      <c r="E20" s="3"/>
-      <c r="F20" s="4"/>
-      <c r="G20" s="4"/>
-    </row>
-    <row r="21" spans="1:7" ht="15.75" customHeight="1">
-      <c r="A21" s="2"/>
-      <c r="B21" s="2"/>
-      <c r="C21" s="3"/>
-      <c r="D21" s="3"/>
-      <c r="E21" s="3"/>
-      <c r="F21" s="4"/>
-      <c r="G21" s="4"/>
-    </row>
-    <row r="22" spans="1:7" ht="15.75" customHeight="1"/>
-    <row r="23" spans="1:7" ht="15.75" customHeight="1"/>
-    <row r="24" spans="1:7" ht="15.75" customHeight="1"/>
-    <row r="25" spans="1:7" ht="15.75" customHeight="1"/>
-    <row r="26" spans="1:7" ht="15.75" customHeight="1"/>
-    <row r="27" spans="1:7" ht="15.75" customHeight="1"/>
-    <row r="28" spans="1:7" ht="15.75" customHeight="1"/>
-    <row r="29" spans="1:7" ht="15.75" customHeight="1"/>
-    <row r="30" spans="1:7" ht="15.75" customHeight="1"/>
-    <row r="31" spans="1:7" ht="15.75" customHeight="1"/>
-    <row r="32" spans="1:7" ht="15.75" customHeight="1"/>
-    <row r="33" ht="15.75" customHeight="1"/>
-    <row r="34" ht="15.75" customHeight="1"/>
-    <row r="35" ht="15.75" customHeight="1"/>
-    <row r="36" ht="15.75" customHeight="1"/>
-    <row r="37" ht="15.75" customHeight="1"/>
-    <row r="38" ht="15.75" customHeight="1"/>
-    <row r="39" ht="15.75" customHeight="1"/>
+    <row r="1" ht="36" customHeight="1">
+      <c r="A1" s="21" t="inlineStr">
+        <is>
+          <t>MATRIZ DE GESTIÓN DE RIESGOS — NOVAFIT ANALYTICS SUITE</t>
+        </is>
+      </c>
+      <c r="K1" s="22" t="n"/>
+      <c r="L1" s="22" t="n"/>
+      <c r="M1" s="22" t="n"/>
+      <c r="N1" s="22" t="n"/>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="23" t="inlineStr">
+        <is>
+          <t>Proyecto: NovaFit Analytics Suite</t>
+        </is>
+      </c>
+      <c r="D2" s="23" t="inlineStr">
+        <is>
+          <t>Fase: Fase 2 — Desarrollo y Construcción</t>
+        </is>
+      </c>
+      <c r="G2" s="23" t="inlineStr">
+        <is>
+          <t>Versión: 2.0 | Fecha: Octubre 2026 | PM: Felipe Romero</t>
+        </is>
+      </c>
+      <c r="K2" s="22" t="n"/>
+      <c r="L2" s="22" t="n"/>
+      <c r="M2" s="22" t="n"/>
+      <c r="N2" s="22" t="n"/>
+    </row>
+    <row r="3" ht="38" customHeight="1">
+      <c r="A3" s="24" t="inlineStr">
+        <is>
+          <t>ID Riesgo</t>
+        </is>
+      </c>
+      <c r="B3" s="24" t="inlineStr">
+        <is>
+          <t>Descripción del Riesgo y Causa Raíz</t>
+        </is>
+      </c>
+      <c r="C3" s="24" t="inlineStr">
+        <is>
+          <t>Categoría</t>
+        </is>
+      </c>
+      <c r="D3" s="24" t="inlineStr">
+        <is>
+          <t>Probabilidad</t>
+        </is>
+      </c>
+      <c r="E3" s="24" t="inlineStr">
+        <is>
+          <t>Impacto</t>
+        </is>
+      </c>
+      <c r="F3" s="24" t="inlineStr">
+        <is>
+          <t>Nivel de Severidad</t>
+        </is>
+      </c>
+      <c r="G3" s="24" t="inlineStr">
+        <is>
+          <t>Acción de Mitigación Proactiva</t>
+        </is>
+      </c>
+      <c r="H3" s="24" t="inlineStr">
+        <is>
+          <t>Plan de Contingencia Reactivo</t>
+        </is>
+      </c>
+      <c r="I3" s="24" t="inlineStr">
+        <is>
+          <t>Responsable</t>
+        </is>
+      </c>
+      <c r="J3" s="24" t="inlineStr">
+        <is>
+          <t>Estado Fase 2</t>
+        </is>
+      </c>
+      <c r="K3" s="22" t="n"/>
+      <c r="L3" s="22" t="n"/>
+      <c r="M3" s="22" t="n"/>
+      <c r="N3" s="22" t="n"/>
+    </row>
+    <row r="4" ht="54" customHeight="1">
+      <c r="A4" s="25" t="inlineStr">
+        <is>
+          <t>RSG-01</t>
+        </is>
+      </c>
+      <c r="B4" s="26" t="inlineStr">
+        <is>
+          <t>Sobrecarga de cómputo en el cálculo retrospectivo ACWR: Latencia excesiva al calcular la ventana móvil de 28 días (carga aguda 7d vs. crónica 28d) ante un gran volumen de series y atletas concurrentes.</t>
+        </is>
+      </c>
+      <c r="C4" s="27" t="inlineStr">
+        <is>
+          <t>Desarrollo</t>
+        </is>
+      </c>
+      <c r="D4" s="27" t="inlineStr">
+        <is>
+          <t>Medio</t>
+        </is>
+      </c>
+      <c r="E4" s="27" t="inlineStr">
+        <is>
+          <t>Crítica</t>
+        </is>
+      </c>
+      <c r="F4" s="28" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="G4" s="26" t="inlineStr">
+        <is>
+          <t>Implementar consultas SQL optimizadas con índices compuestos en (athlete_id, workout_date), cálculo asíncrono en FastAPI y almacenamiento en caché en memoria.</t>
+        </is>
+      </c>
+      <c r="H4" s="26" t="inlineStr">
+        <is>
+          <t>Si la latencia supera 1.5s, degradar a cálculo nocturno por lote (cron job) almacenando los ratios en la tabla acwr_records.</t>
+        </is>
+      </c>
+      <c r="I4" s="27" t="inlineStr">
+        <is>
+          <t>Vicente Gilbert</t>
+        </is>
+      </c>
+      <c r="J4" s="29" t="inlineStr">
+        <is>
+          <t>Mitigado</t>
+        </is>
+      </c>
+      <c r="K4" s="22" t="n"/>
+      <c r="L4" s="22" t="n"/>
+      <c r="M4" s="22" t="n"/>
+      <c r="N4" s="22" t="n"/>
+    </row>
+    <row r="5" ht="54" customHeight="1">
+      <c r="A5" s="30" t="inlineStr">
+        <is>
+          <t>RSG-02</t>
+        </is>
+      </c>
+      <c r="B5" s="31" t="inlineStr">
+        <is>
+          <t>Desincronización de datos móviles en zonas con baja conectividad: Pérdida de registros de series si el atleta entrena en zonas del gimnasio o subterráneos sin cobertura celular ni Wi-Fi.</t>
+        </is>
+      </c>
+      <c r="C5" s="32" t="inlineStr">
+        <is>
+          <t>Desarrollo</t>
+        </is>
+      </c>
+      <c r="D5" s="32" t="inlineStr">
+        <is>
+          <t>Medio</t>
+        </is>
+      </c>
+      <c r="E5" s="32" t="inlineStr">
+        <is>
+          <t>Crítica</t>
+        </is>
+      </c>
+      <c r="F5" s="28" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="G5" s="31" t="inlineStr">
+        <is>
+          <t>Implementar arquitectura offline-first con almacenamiento local en SQLite/AsyncStorage (React Native) y cola de sincronización automática al recuperar conexión.</t>
+        </is>
+      </c>
+      <c r="H5" s="31" t="inlineStr">
+        <is>
+          <t>Exportar copia local en JSON temporal en el dispositivo del atleta y emitir aviso visual de 'Datos pendientes de sincronizar'.</t>
+        </is>
+      </c>
+      <c r="I5" s="32" t="inlineStr">
+        <is>
+          <t>Antonio Maturana</t>
+        </is>
+      </c>
+      <c r="J5" s="29" t="inlineStr">
+        <is>
+          <t>Mitigado</t>
+        </is>
+      </c>
+      <c r="K5" s="22" t="n"/>
+      <c r="L5" s="22" t="n"/>
+      <c r="M5" s="22" t="n"/>
+      <c r="N5" s="22" t="n"/>
+    </row>
+    <row r="6" ht="54" customHeight="1">
+      <c r="A6" s="25" t="inlineStr">
+        <is>
+          <t>RSG-03</t>
+        </is>
+      </c>
+      <c r="B6" s="26" t="inlineStr">
+        <is>
+          <t>Inconsistencia relacional en datos transaccionales contables: Conflictos, duplicidades o datos huérfanos al registrar suscripciones, facturación y pagos concurrentes.</t>
+        </is>
+      </c>
+      <c r="C6" s="27" t="inlineStr">
+        <is>
+          <t>Desarrollo</t>
+        </is>
+      </c>
+      <c r="D6" s="27" t="inlineStr">
+        <is>
+          <t>Bajo</t>
+        </is>
+      </c>
+      <c r="E6" s="27" t="inlineStr">
+        <is>
+          <t>Crítica</t>
+        </is>
+      </c>
+      <c r="F6" s="33" t="inlineStr">
+        <is>
+          <t>Medio</t>
+        </is>
+      </c>
+      <c r="G6" s="26" t="inlineStr">
+        <is>
+          <t>Aplicar migraciones versionadas con Alembic, restricciones de clave foránea e integridad referencial estricta, y transacciones atómicas ACID en PostgreSQL con ON DELETE RESTRICT.</t>
+        </is>
+      </c>
+      <c r="H6" s="26" t="inlineStr">
+        <is>
+          <t>Rollback inmediato de la transacción ante excepciones de base de datos y registro de auditoría en logs estructurados.</t>
+        </is>
+      </c>
+      <c r="I6" s="27" t="inlineStr">
+        <is>
+          <t>Yulian Silva</t>
+        </is>
+      </c>
+      <c r="J6" s="29" t="inlineStr">
+        <is>
+          <t>Mitigado</t>
+        </is>
+      </c>
+      <c r="K6" s="22" t="n"/>
+      <c r="L6" s="22" t="n"/>
+      <c r="M6" s="22" t="n"/>
+      <c r="N6" s="22" t="n"/>
+    </row>
+    <row r="7" ht="54" customHeight="1">
+      <c r="A7" s="30" t="inlineStr">
+        <is>
+          <t>RSG-04</t>
+        </is>
+      </c>
+      <c r="B7" s="31" t="inlineStr">
+        <is>
+          <t>Vulnerabilidades de seguridad en endpoints y fuga de datos: Exposición indebida de datos médicos/antropométricos de atletas o vulnerabilidad en autenticación de la API REST.</t>
+        </is>
+      </c>
+      <c r="C7" s="32" t="inlineStr">
+        <is>
+          <t>Seguridad</t>
+        </is>
+      </c>
+      <c r="D7" s="32" t="inlineStr">
+        <is>
+          <t>Bajo</t>
+        </is>
+      </c>
+      <c r="E7" s="32" t="inlineStr">
+        <is>
+          <t>Catastrófica</t>
+        </is>
+      </c>
+      <c r="F7" s="28" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="G7" s="31" t="inlineStr">
+        <is>
+          <t>Uso de hashing Bcrypt para contraseñas, tokens JWT con tiempo de expiración corto, validación estricta de esquemas Pydantic, consultas parametrizadas y CORS restringido.</t>
+        </is>
+      </c>
+      <c r="H7" s="31" t="inlineStr">
+        <is>
+          <t>Revocación masiva inmediata de tokens JWT mediante lista negra en caché y forzar restablecimiento seguro de credenciales.</t>
+        </is>
+      </c>
+      <c r="I7" s="32" t="inlineStr">
+        <is>
+          <t>Vicente Gilbert</t>
+        </is>
+      </c>
+      <c r="J7" s="29" t="inlineStr">
+        <is>
+          <t>Mitigado</t>
+        </is>
+      </c>
+      <c r="K7" s="22" t="n"/>
+      <c r="L7" s="22" t="n"/>
+      <c r="M7" s="22" t="n"/>
+      <c r="N7" s="22" t="n"/>
+    </row>
+    <row r="8" ht="54" customHeight="1">
+      <c r="A8" s="25" t="inlineStr">
+        <is>
+          <t>RSG-05</t>
+        </is>
+      </c>
+      <c r="B8" s="26" t="inlineStr">
+        <is>
+          <t>Fricción y lentitud en la carga de series por parte del atleta: Abandono del uso de la app móvil si el proceso de ingreso de pesos y repeticiones resulta engorroso durante el entrenamiento físico.</t>
+        </is>
+      </c>
+      <c r="C8" s="27" t="inlineStr">
+        <is>
+          <t>Desarrollo</t>
+        </is>
+      </c>
+      <c r="D8" s="27" t="inlineStr">
+        <is>
+          <t>Medio</t>
+        </is>
+      </c>
+      <c r="E8" s="27" t="inlineStr">
+        <is>
+          <t>Marginal</t>
+        </is>
+      </c>
+      <c r="F8" s="33" t="inlineStr">
+        <is>
+          <t>Medio</t>
+        </is>
+      </c>
+      <c r="G8" s="26" t="inlineStr">
+        <is>
+          <t>Diseñar interfaz minimalista con función de autocompletado inteligente (Auto-Fill) basado en la última sesión, botones táctiles grandes y modo oscuro de alto contraste.</t>
+        </is>
+      </c>
+      <c r="H8" s="26" t="inlineStr">
+        <is>
+          <t>Habilitar modo de registro rápido por serie con gestos rápidos y confirmación táctil (haptic feedback).</t>
+        </is>
+      </c>
+      <c r="I8" s="27" t="inlineStr">
+        <is>
+          <t>Antonio Maturana</t>
+        </is>
+      </c>
+      <c r="J8" s="29" t="inlineStr">
+        <is>
+          <t>Mitigado</t>
+        </is>
+      </c>
+      <c r="K8" s="22" t="n"/>
+      <c r="L8" s="22" t="n"/>
+      <c r="M8" s="22" t="n"/>
+      <c r="N8" s="22" t="n"/>
+    </row>
+    <row r="9" ht="54" customHeight="1">
+      <c r="A9" s="30" t="inlineStr">
+        <is>
+          <t>RSG-06</t>
+        </is>
+      </c>
+      <c r="B9" s="31" t="inlineStr">
+        <is>
+          <t>Fallas, latencia o pérdida de eventos en Webhooks de Mercado Pago: Pérdida o demora en la confirmación de pagos de membresías debido a timeouts o indisponibilidad temporal del proveedor externo.</t>
+        </is>
+      </c>
+      <c r="C9" s="32" t="inlineStr">
+        <is>
+          <t>Externo</t>
+        </is>
+      </c>
+      <c r="D9" s="32" t="inlineStr">
+        <is>
+          <t>Medio</t>
+        </is>
+      </c>
+      <c r="E9" s="32" t="inlineStr">
+        <is>
+          <t>Crítica</t>
+        </is>
+      </c>
+      <c r="F9" s="28" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="G9" s="31" t="inlineStr">
+        <is>
+          <t>Implementar endpoints webhook idempotentes en FastAPI con registro de auditoría en base de datos, reintentos automáticos con backoff exponencial y verificación manual vía polling API.</t>
+        </is>
+      </c>
+      <c r="H9" s="31" t="inlineStr">
+        <is>
+          <t>Ejecutar proceso de conciliación bancaria manual desde el panel web con el botón 'Sincronizar estado MP' mediante consulta directa por Payment ID.</t>
+        </is>
+      </c>
+      <c r="I9" s="32" t="inlineStr">
+        <is>
+          <t>Vicente Gilbert</t>
+        </is>
+      </c>
+      <c r="J9" s="29" t="inlineStr">
+        <is>
+          <t>Mitigado</t>
+        </is>
+      </c>
+      <c r="K9" s="22" t="n"/>
+      <c r="L9" s="22" t="n"/>
+      <c r="M9" s="22" t="n"/>
+      <c r="N9" s="22" t="n"/>
+    </row>
+    <row r="10" ht="54" customHeight="1">
+      <c r="A10" s="25" t="inlineStr">
+        <is>
+          <t>RSG-07</t>
+        </is>
+      </c>
+      <c r="B10" s="26" t="inlineStr">
+        <is>
+          <t>Límites de cuota o tiempos de arranque en frío (Cold Starts) en servicios Cloud: Demoras de hasta 40 segundos en las primeras peticiones por suspensión de instancias gratuitas en Render.</t>
+        </is>
+      </c>
+      <c r="C10" s="27" t="inlineStr">
+        <is>
+          <t>Externo</t>
+        </is>
+      </c>
+      <c r="D10" s="27" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="E10" s="27" t="inlineStr">
+        <is>
+          <t>Marginal</t>
+        </is>
+      </c>
+      <c r="F10" s="33" t="inlineStr">
+        <is>
+          <t>Medio</t>
+        </is>
+      </c>
+      <c r="G10" s="26" t="inlineStr">
+        <is>
+          <t>Configurar componente ServerWakeUp en web y móvil con indicador visual amigable, y programar peticiones periódicas de calentamiento (keep-alive) mediante cron automatizado.</t>
+        </is>
+      </c>
+      <c r="H10" s="26" t="inlineStr">
+        <is>
+          <t>Mostrar al usuario pantalla de carga explicativa indicando 'Conectando con servidores NovaFit...' sin bloquear la navegación offline.</t>
+        </is>
+      </c>
+      <c r="I10" s="27" t="inlineStr">
+        <is>
+          <t>Vicente Gilbert</t>
+        </is>
+      </c>
+      <c r="J10" s="29" t="inlineStr">
+        <is>
+          <t>Mitigado</t>
+        </is>
+      </c>
+      <c r="K10" s="22" t="n"/>
+      <c r="L10" s="22" t="n"/>
+      <c r="M10" s="22" t="n"/>
+      <c r="N10" s="22" t="n"/>
+    </row>
+    <row r="11" ht="54" customHeight="1">
+      <c r="A11" s="30" t="inlineStr">
+        <is>
+          <t>RSG-08</t>
+        </is>
+      </c>
+      <c r="B11" s="31" t="inlineStr">
+        <is>
+          <t>Incompatibilidad por actualización de dependencias de terceros: Ruptura de builds en React Native / Expo SDK o paquetes de Node.js / Python por releases no controlados.</t>
+        </is>
+      </c>
+      <c r="C11" s="32" t="inlineStr">
+        <is>
+          <t>Externo</t>
+        </is>
+      </c>
+      <c r="D11" s="32" t="inlineStr">
+        <is>
+          <t>Bajo</t>
+        </is>
+      </c>
+      <c r="E11" s="32" t="inlineStr">
+        <is>
+          <t>Marginal</t>
+        </is>
+      </c>
+      <c r="F11" s="29" t="inlineStr">
+        <is>
+          <t>Bajo</t>
+        </is>
+      </c>
+      <c r="G11" s="31" t="inlineStr">
+        <is>
+          <t>Congelar versiones exactas de librerías mediante package-lock.json y requirements.txt, prohibiendo actualizaciones de versión mayor (major) durante la Fase 2.</t>
+        </is>
+      </c>
+      <c r="H11" s="31" t="inlineStr">
+        <is>
+          <t>Restaurar el entorno de desarrollo a partir del commit estable etiquetado en Git y levantar contenedores Docker limpios.</t>
+        </is>
+      </c>
+      <c r="I11" s="32" t="inlineStr">
+        <is>
+          <t>Antonio Maturana</t>
+        </is>
+      </c>
+      <c r="J11" s="29" t="inlineStr">
+        <is>
+          <t>Mitigado</t>
+        </is>
+      </c>
+      <c r="K11" s="22" t="n"/>
+      <c r="L11" s="22" t="n"/>
+      <c r="M11" s="22" t="n"/>
+      <c r="N11" s="22" t="n"/>
+    </row>
+    <row r="12" ht="54" customHeight="1">
+      <c r="A12" s="25" t="inlineStr">
+        <is>
+          <t>RSG-09</t>
+        </is>
+      </c>
+      <c r="B12" s="26" t="inlineStr">
+        <is>
+          <t>Desfase en la integración entre Frontend y Backend: Retrasos en las entregas de sprint por divergencias entre los tipos de datos que espera el cliente web/móvil y los esquemas JSON de la API.</t>
+        </is>
+      </c>
+      <c r="C12" s="27" t="inlineStr">
+        <is>
+          <t>Proyecto</t>
+        </is>
+      </c>
+      <c r="D12" s="27" t="inlineStr">
+        <is>
+          <t>Medio</t>
+        </is>
+      </c>
+      <c r="E12" s="27" t="inlineStr">
+        <is>
+          <t>Crítica</t>
+        </is>
+      </c>
+      <c r="F12" s="28" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="G12" s="26" t="inlineStr">
+        <is>
+          <t>Diseñar y congelar contratos de interfaz tempranos mediante la documentación interactiva Swagger/OpenAPI de FastAPI antes de comenzar la codificación de vistas.</t>
+        </is>
+      </c>
+      <c r="H12" s="26" t="inlineStr">
+        <is>
+          <t>Sesiones semanales obligatorias de alineación técnica entre el desarrollador Backend y Frontend para revisión conjunta de payloads JSON.</t>
+        </is>
+      </c>
+      <c r="I12" s="27" t="inlineStr">
+        <is>
+          <t>Felipe Romero</t>
+        </is>
+      </c>
+      <c r="J12" s="29" t="inlineStr">
+        <is>
+          <t>Mitigado</t>
+        </is>
+      </c>
+      <c r="K12" s="22" t="n"/>
+      <c r="L12" s="22" t="n"/>
+      <c r="M12" s="22" t="n"/>
+      <c r="N12" s="22" t="n"/>
+    </row>
+    <row r="13" ht="54" customHeight="1">
+      <c r="A13" s="30" t="inlineStr">
+        <is>
+          <t>RSG-10</t>
+        </is>
+      </c>
+      <c r="B13" s="31" t="inlineStr">
+        <is>
+          <t>Detección tardía de errores en flujos críticos previo a entregas: Acumulación de bugs no detectados que impidan la demostración funcional en el Hito de Avance y Cierre de Fase 2.</t>
+        </is>
+      </c>
+      <c r="C13" s="32" t="inlineStr">
+        <is>
+          <t>Proyecto</t>
+        </is>
+      </c>
+      <c r="D13" s="32" t="inlineStr">
+        <is>
+          <t>Medio</t>
+        </is>
+      </c>
+      <c r="E13" s="32" t="inlineStr">
+        <is>
+          <t>Crítica</t>
+        </is>
+      </c>
+      <c r="F13" s="28" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="G13" s="31" t="inlineStr">
+        <is>
+          <t>Ejecución continua de los 16 casos de prueba del Plan de Pruebas de Software NovaFit y establecimiento de un Code Freeze de 3 días antes de cada cierre de hito para testing de QA.</t>
+        </is>
+      </c>
+      <c r="H13" s="31" t="inlineStr">
+        <is>
+          <t>Jornada de depuración intensiva priorizando los casos P1 (Autenticación, Facturación Mercado Pago y Motor ACWR).</t>
+        </is>
+      </c>
+      <c r="I13" s="32" t="inlineStr">
+        <is>
+          <t>Steven San Martín</t>
+        </is>
+      </c>
+      <c r="J13" s="29" t="inlineStr">
+        <is>
+          <t>Mitigado</t>
+        </is>
+      </c>
+      <c r="K13" s="22" t="n"/>
+      <c r="L13" s="22" t="n"/>
+      <c r="M13" s="22" t="n"/>
+      <c r="N13" s="22" t="n"/>
+    </row>
+    <row r="14" ht="54" customHeight="1">
+      <c r="A14" s="25" t="inlineStr">
+        <is>
+          <t>RSG-11</t>
+        </is>
+      </c>
+      <c r="B14" s="26" t="inlineStr">
+        <is>
+          <t>Desviación de alcance respecto al ERS de la Fase 1: Incorporación descontrolada de requerimientos adicionales fuera de plazo que afecten el cumplimiento de la Carta Gantt.</t>
+        </is>
+      </c>
+      <c r="C14" s="27" t="inlineStr">
+        <is>
+          <t>Proyecto</t>
+        </is>
+      </c>
+      <c r="D14" s="27" t="inlineStr">
+        <is>
+          <t>Bajo</t>
+        </is>
+      </c>
+      <c r="E14" s="27" t="inlineStr">
+        <is>
+          <t>Marginal</t>
+        </is>
+      </c>
+      <c r="F14" s="29" t="inlineStr">
+        <is>
+          <t>Bajo</t>
+        </is>
+      </c>
+      <c r="G14" s="26" t="inlineStr">
+        <is>
+          <t>Canalización obligatoria de cualquier modificación a través de la Matriz de Control de Cambios, evaluando su impacto en días y esfuerzo antes de ser aprobada por el PM.</t>
+        </is>
+      </c>
+      <c r="H14" s="26" t="inlineStr">
+        <is>
+          <t>Rechazar o postergar para Fase 3 (o versión 2.0 comercial) todo requerimiento no esencial para la validación de la tesis.</t>
+        </is>
+      </c>
+      <c r="I14" s="27" t="inlineStr">
+        <is>
+          <t>Felipe Romero</t>
+        </is>
+      </c>
+      <c r="J14" s="29" t="inlineStr">
+        <is>
+          <t>Mitigado</t>
+        </is>
+      </c>
+      <c r="K14" s="22" t="n"/>
+      <c r="L14" s="22" t="n"/>
+      <c r="M14" s="22" t="n"/>
+      <c r="N14" s="22" t="n"/>
+    </row>
+    <row r="15" ht="54" customHeight="1">
+      <c r="A15" s="30" t="inlineStr">
+        <is>
+          <t>RSG-12</t>
+        </is>
+      </c>
+      <c r="B15" s="31" t="inlineStr">
+        <is>
+          <t>Indisponibilidad fortuita de algún integrante del equipo: Retrasos imprevistos por motivos de salud, cortes de servicio o fuerza mayor de algún miembro del grupo.</t>
+        </is>
+      </c>
+      <c r="C15" s="32" t="inlineStr">
+        <is>
+          <t>Proyecto</t>
+        </is>
+      </c>
+      <c r="D15" s="32" t="inlineStr">
+        <is>
+          <t>Bajo</t>
+        </is>
+      </c>
+      <c r="E15" s="32" t="inlineStr">
+        <is>
+          <t>Marginal</t>
+        </is>
+      </c>
+      <c r="F15" s="29" t="inlineStr">
+        <is>
+          <t>Bajo</t>
+        </is>
+      </c>
+      <c r="G15" s="31" t="inlineStr">
+        <is>
+          <t>Respaldo diario de código y ramas en GitHub bajo metodología GitFlow, asignación de roles de soporte técnico secundario según la Matriz RACI y minutas al día.</t>
+        </is>
+      </c>
+      <c r="H15" s="31" t="inlineStr">
+        <is>
+          <t>Reasignación temporal de tareas críticas hacia el Tech Lead (Felipe Romero) con redistribución de tickets en Jira/Trello.</t>
+        </is>
+      </c>
+      <c r="I15" s="32" t="inlineStr">
+        <is>
+          <t>Felipe Romero</t>
+        </is>
+      </c>
+      <c r="J15" s="29" t="inlineStr">
+        <is>
+          <t>Mitigado</t>
+        </is>
+      </c>
+      <c r="K15" s="22" t="n"/>
+      <c r="L15" s="22" t="n"/>
+      <c r="M15" s="22" t="n"/>
+      <c r="N15" s="22" t="n"/>
+    </row>
+    <row r="16" ht="24" customHeight="1">
+      <c r="A16" s="34" t="inlineStr">
+        <is>
+          <t>Total de Riesgos Gestionados: 12  |  Mitigados al Cierre Fase 2: 12 (100%)</t>
+        </is>
+      </c>
+      <c r="F16" s="35" t="n"/>
+      <c r="G16" s="35" t="n"/>
+      <c r="H16" s="36" t="n"/>
+      <c r="I16" s="36" t="n"/>
+      <c r="J16" s="36" t="n"/>
+      <c r="K16" s="22" t="n"/>
+      <c r="L16" s="22" t="n"/>
+      <c r="M16" s="22" t="n"/>
+      <c r="N16" s="22" t="n"/>
+    </row>
+    <row r="17" ht="15.75" customHeight="1">
+      <c r="A17" s="37" t="n"/>
+      <c r="B17" s="37" t="n"/>
+      <c r="C17" s="38" t="n"/>
+      <c r="D17" s="38" t="n"/>
+      <c r="E17" s="38" t="n"/>
+      <c r="F17" s="37" t="n"/>
+      <c r="G17" s="37" t="n"/>
+      <c r="H17" s="22" t="n"/>
+      <c r="I17" s="22" t="n"/>
+      <c r="J17" s="22" t="n"/>
+      <c r="K17" s="22" t="n"/>
+      <c r="L17" s="22" t="n"/>
+      <c r="M17" s="22" t="n"/>
+      <c r="N17" s="22" t="n"/>
+    </row>
+    <row r="18" ht="15.75" customHeight="1">
+      <c r="A18" s="37" t="n"/>
+      <c r="B18" s="37" t="n"/>
+      <c r="C18" s="38" t="n"/>
+      <c r="D18" s="38" t="n"/>
+      <c r="E18" s="38" t="n"/>
+      <c r="F18" s="37" t="n"/>
+      <c r="G18" s="37" t="n"/>
+      <c r="H18" s="22" t="n"/>
+      <c r="I18" s="22" t="n"/>
+      <c r="J18" s="22" t="n"/>
+      <c r="K18" s="22" t="n"/>
+      <c r="L18" s="22" t="n"/>
+      <c r="M18" s="22" t="n"/>
+      <c r="N18" s="22" t="n"/>
+    </row>
+    <row r="19" ht="15.75" customHeight="1">
+      <c r="A19" s="37" t="n"/>
+      <c r="B19" s="37" t="n"/>
+      <c r="C19" s="38" t="n"/>
+      <c r="D19" s="38" t="n"/>
+      <c r="E19" s="38" t="n"/>
+      <c r="F19" s="37" t="n"/>
+      <c r="G19" s="37" t="n"/>
+      <c r="H19" s="22" t="n"/>
+      <c r="I19" s="22" t="n"/>
+      <c r="J19" s="22" t="n"/>
+      <c r="K19" s="22" t="n"/>
+      <c r="L19" s="22" t="n"/>
+      <c r="M19" s="22" t="n"/>
+      <c r="N19" s="22" t="n"/>
+    </row>
+    <row r="20" ht="15.75" customHeight="1">
+      <c r="A20" s="37" t="n"/>
+      <c r="B20" s="37" t="n"/>
+      <c r="C20" s="38" t="n"/>
+      <c r="D20" s="38" t="n"/>
+      <c r="E20" s="38" t="n"/>
+      <c r="F20" s="37" t="n"/>
+      <c r="G20" s="37" t="n"/>
+      <c r="H20" s="22" t="n"/>
+      <c r="I20" s="22" t="n"/>
+      <c r="J20" s="22" t="n"/>
+      <c r="K20" s="22" t="n"/>
+      <c r="L20" s="22" t="n"/>
+      <c r="M20" s="22" t="n"/>
+      <c r="N20" s="22" t="n"/>
+    </row>
+    <row r="21" ht="15.75" customHeight="1">
+      <c r="A21" s="37" t="n"/>
+      <c r="B21" s="37" t="n"/>
+      <c r="C21" s="38" t="n"/>
+      <c r="D21" s="38" t="n"/>
+      <c r="E21" s="38" t="n"/>
+      <c r="F21" s="37" t="n"/>
+      <c r="G21" s="37" t="n"/>
+      <c r="H21" s="22" t="n"/>
+      <c r="I21" s="22" t="n"/>
+      <c r="J21" s="22" t="n"/>
+      <c r="K21" s="22" t="n"/>
+      <c r="L21" s="22" t="n"/>
+      <c r="M21" s="22" t="n"/>
+      <c r="N21" s="22" t="n"/>
+    </row>
+    <row r="22" ht="15.75" customHeight="1">
+      <c r="A22" s="22" t="n"/>
+      <c r="B22" s="22" t="n"/>
+      <c r="C22" s="22" t="n"/>
+      <c r="D22" s="22" t="n"/>
+      <c r="E22" s="22" t="n"/>
+      <c r="F22" s="22" t="n"/>
+      <c r="G22" s="22" t="n"/>
+      <c r="H22" s="22" t="n"/>
+      <c r="I22" s="22" t="n"/>
+      <c r="J22" s="22" t="n"/>
+      <c r="K22" s="22" t="n"/>
+      <c r="L22" s="22" t="n"/>
+      <c r="M22" s="22" t="n"/>
+      <c r="N22" s="22" t="n"/>
+    </row>
+    <row r="23" ht="15.75" customHeight="1">
+      <c r="A23" s="22" t="n"/>
+      <c r="B23" s="22" t="n"/>
+      <c r="C23" s="22" t="n"/>
+      <c r="D23" s="22" t="n"/>
+      <c r="E23" s="22" t="n"/>
+      <c r="F23" s="22" t="n"/>
+      <c r="G23" s="22" t="n"/>
+      <c r="H23" s="22" t="n"/>
+      <c r="I23" s="22" t="n"/>
+      <c r="J23" s="22" t="n"/>
+      <c r="K23" s="22" t="n"/>
+      <c r="L23" s="22" t="n"/>
+      <c r="M23" s="22" t="n"/>
+      <c r="N23" s="22" t="n"/>
+    </row>
+    <row r="24" ht="15.75" customHeight="1">
+      <c r="A24" s="22" t="n"/>
+      <c r="B24" s="22" t="n"/>
+      <c r="C24" s="22" t="n"/>
+      <c r="D24" s="22" t="n"/>
+      <c r="E24" s="22" t="n"/>
+      <c r="F24" s="22" t="n"/>
+      <c r="G24" s="22" t="n"/>
+      <c r="H24" s="22" t="n"/>
+      <c r="I24" s="22" t="n"/>
+      <c r="J24" s="22" t="n"/>
+      <c r="K24" s="22" t="n"/>
+      <c r="L24" s="22" t="n"/>
+      <c r="M24" s="22" t="n"/>
+      <c r="N24" s="22" t="n"/>
+    </row>
+    <row r="25" ht="15.75" customHeight="1">
+      <c r="A25" s="22" t="n"/>
+      <c r="B25" s="22" t="n"/>
+      <c r="C25" s="22" t="n"/>
+      <c r="D25" s="22" t="n"/>
+      <c r="E25" s="22" t="n"/>
+      <c r="F25" s="22" t="n"/>
+      <c r="G25" s="22" t="n"/>
+      <c r="H25" s="22" t="n"/>
+      <c r="I25" s="22" t="n"/>
+      <c r="J25" s="22" t="n"/>
+      <c r="K25" s="22" t="n"/>
+      <c r="L25" s="22" t="n"/>
+      <c r="M25" s="22" t="n"/>
+      <c r="N25" s="22" t="n"/>
+    </row>
+    <row r="26" ht="15.75" customHeight="1">
+      <c r="A26" s="22" t="n"/>
+      <c r="B26" s="22" t="n"/>
+      <c r="C26" s="22" t="n"/>
+      <c r="D26" s="22" t="n"/>
+      <c r="E26" s="22" t="n"/>
+      <c r="F26" s="22" t="n"/>
+      <c r="G26" s="22" t="n"/>
+      <c r="H26" s="22" t="n"/>
+      <c r="I26" s="22" t="n"/>
+      <c r="J26" s="22" t="n"/>
+      <c r="K26" s="22" t="n"/>
+      <c r="L26" s="22" t="n"/>
+      <c r="M26" s="22" t="n"/>
+      <c r="N26" s="22" t="n"/>
+    </row>
+    <row r="27" ht="15.75" customHeight="1">
+      <c r="A27" s="22" t="n"/>
+      <c r="B27" s="22" t="n"/>
+      <c r="C27" s="22" t="n"/>
+      <c r="D27" s="22" t="n"/>
+      <c r="E27" s="22" t="n"/>
+      <c r="F27" s="22" t="n"/>
+      <c r="G27" s="22" t="n"/>
+      <c r="H27" s="22" t="n"/>
+      <c r="I27" s="22" t="n"/>
+      <c r="J27" s="22" t="n"/>
+      <c r="K27" s="22" t="n"/>
+      <c r="L27" s="22" t="n"/>
+      <c r="M27" s="22" t="n"/>
+      <c r="N27" s="22" t="n"/>
+    </row>
+    <row r="28" ht="15.75" customHeight="1">
+      <c r="A28" s="22" t="n"/>
+      <c r="B28" s="22" t="n"/>
+      <c r="C28" s="22" t="n"/>
+      <c r="D28" s="22" t="n"/>
+      <c r="E28" s="22" t="n"/>
+      <c r="F28" s="22" t="n"/>
+      <c r="G28" s="22" t="n"/>
+      <c r="H28" s="22" t="n"/>
+      <c r="I28" s="22" t="n"/>
+      <c r="J28" s="22" t="n"/>
+      <c r="K28" s="22" t="n"/>
+      <c r="L28" s="22" t="n"/>
+      <c r="M28" s="22" t="n"/>
+      <c r="N28" s="22" t="n"/>
+    </row>
+    <row r="29" ht="15.75" customHeight="1">
+      <c r="A29" s="22" t="n"/>
+      <c r="B29" s="22" t="n"/>
+      <c r="C29" s="22" t="n"/>
+      <c r="D29" s="22" t="n"/>
+      <c r="E29" s="22" t="n"/>
+      <c r="F29" s="22" t="n"/>
+      <c r="G29" s="22" t="n"/>
+      <c r="H29" s="22" t="n"/>
+      <c r="I29" s="22" t="n"/>
+      <c r="J29" s="22" t="n"/>
+      <c r="K29" s="22" t="n"/>
+      <c r="L29" s="22" t="n"/>
+      <c r="M29" s="22" t="n"/>
+      <c r="N29" s="22" t="n"/>
+    </row>
+    <row r="30" ht="15.75" customHeight="1">
+      <c r="A30" s="22" t="n"/>
+      <c r="B30" s="22" t="n"/>
+      <c r="C30" s="22" t="n"/>
+      <c r="D30" s="22" t="n"/>
+      <c r="E30" s="22" t="n"/>
+      <c r="F30" s="22" t="n"/>
+      <c r="G30" s="22" t="n"/>
+      <c r="H30" s="22" t="n"/>
+      <c r="I30" s="22" t="n"/>
+      <c r="J30" s="22" t="n"/>
+      <c r="K30" s="22" t="n"/>
+      <c r="L30" s="22" t="n"/>
+      <c r="M30" s="22" t="n"/>
+      <c r="N30" s="22" t="n"/>
+    </row>
+    <row r="31" ht="15.75" customHeight="1">
+      <c r="A31" s="22" t="n"/>
+      <c r="B31" s="22" t="n"/>
+      <c r="C31" s="22" t="n"/>
+      <c r="D31" s="22" t="n"/>
+      <c r="E31" s="22" t="n"/>
+      <c r="F31" s="22" t="n"/>
+      <c r="G31" s="22" t="n"/>
+      <c r="H31" s="22" t="n"/>
+      <c r="I31" s="22" t="n"/>
+      <c r="J31" s="22" t="n"/>
+      <c r="K31" s="22" t="n"/>
+      <c r="L31" s="22" t="n"/>
+      <c r="M31" s="22" t="n"/>
+      <c r="N31" s="22" t="n"/>
+    </row>
+    <row r="32" ht="15.75" customHeight="1">
+      <c r="A32" s="22" t="n"/>
+      <c r="B32" s="22" t="n"/>
+      <c r="C32" s="22" t="n"/>
+      <c r="D32" s="22" t="n"/>
+      <c r="E32" s="22" t="n"/>
+      <c r="F32" s="22" t="n"/>
+      <c r="G32" s="22" t="n"/>
+      <c r="H32" s="22" t="n"/>
+      <c r="I32" s="22" t="n"/>
+      <c r="J32" s="22" t="n"/>
+      <c r="K32" s="22" t="n"/>
+      <c r="L32" s="22" t="n"/>
+      <c r="M32" s="22" t="n"/>
+      <c r="N32" s="22" t="n"/>
+    </row>
+    <row r="33" ht="15.75" customHeight="1">
+      <c r="A33" s="22" t="n"/>
+      <c r="B33" s="22" t="n"/>
+      <c r="C33" s="22" t="n"/>
+      <c r="D33" s="22" t="n"/>
+      <c r="E33" s="22" t="n"/>
+      <c r="F33" s="22" t="n"/>
+      <c r="G33" s="22" t="n"/>
+      <c r="H33" s="22" t="n"/>
+      <c r="I33" s="22" t="n"/>
+      <c r="J33" s="22" t="n"/>
+      <c r="K33" s="22" t="n"/>
+      <c r="L33" s="22" t="n"/>
+      <c r="M33" s="22" t="n"/>
+      <c r="N33" s="22" t="n"/>
+    </row>
+    <row r="34" ht="15.75" customHeight="1">
+      <c r="A34" s="22" t="n"/>
+      <c r="B34" s="22" t="n"/>
+      <c r="C34" s="22" t="n"/>
+      <c r="D34" s="22" t="n"/>
+      <c r="E34" s="22" t="n"/>
+      <c r="F34" s="22" t="n"/>
+      <c r="G34" s="22" t="n"/>
+      <c r="H34" s="22" t="n"/>
+      <c r="I34" s="22" t="n"/>
+      <c r="J34" s="22" t="n"/>
+      <c r="K34" s="22" t="n"/>
+      <c r="L34" s="22" t="n"/>
+      <c r="M34" s="22" t="n"/>
+      <c r="N34" s="22" t="n"/>
+    </row>
+    <row r="35" ht="15.75" customHeight="1">
+      <c r="A35" s="22" t="n"/>
+      <c r="B35" s="22" t="n"/>
+      <c r="C35" s="22" t="n"/>
+      <c r="D35" s="22" t="n"/>
+      <c r="E35" s="22" t="n"/>
+      <c r="F35" s="22" t="n"/>
+      <c r="G35" s="22" t="n"/>
+      <c r="H35" s="22" t="n"/>
+      <c r="I35" s="22" t="n"/>
+      <c r="J35" s="22" t="n"/>
+      <c r="K35" s="22" t="n"/>
+      <c r="L35" s="22" t="n"/>
+      <c r="M35" s="22" t="n"/>
+      <c r="N35" s="22" t="n"/>
+    </row>
+    <row r="36" ht="15.75" customHeight="1">
+      <c r="A36" s="22" t="n"/>
+      <c r="B36" s="22" t="n"/>
+      <c r="C36" s="22" t="n"/>
+      <c r="D36" s="22" t="n"/>
+      <c r="E36" s="22" t="n"/>
+      <c r="F36" s="22" t="n"/>
+      <c r="G36" s="22" t="n"/>
+      <c r="H36" s="22" t="n"/>
+      <c r="I36" s="22" t="n"/>
+      <c r="J36" s="22" t="n"/>
+      <c r="K36" s="22" t="n"/>
+      <c r="L36" s="22" t="n"/>
+      <c r="M36" s="22" t="n"/>
+      <c r="N36" s="22" t="n"/>
+    </row>
+    <row r="37" ht="15.75" customHeight="1">
+      <c r="A37" s="22" t="n"/>
+      <c r="B37" s="22" t="n"/>
+      <c r="C37" s="22" t="n"/>
+      <c r="D37" s="22" t="n"/>
+      <c r="E37" s="22" t="n"/>
+      <c r="F37" s="22" t="n"/>
+      <c r="G37" s="22" t="n"/>
+      <c r="H37" s="22" t="n"/>
+      <c r="I37" s="22" t="n"/>
+      <c r="J37" s="22" t="n"/>
+      <c r="K37" s="22" t="n"/>
+      <c r="L37" s="22" t="n"/>
+      <c r="M37" s="22" t="n"/>
+      <c r="N37" s="22" t="n"/>
+    </row>
+    <row r="38" ht="15.75" customHeight="1">
+      <c r="A38" s="22" t="n"/>
+      <c r="B38" s="22" t="n"/>
+      <c r="C38" s="22" t="n"/>
+      <c r="D38" s="22" t="n"/>
+      <c r="E38" s="22" t="n"/>
+      <c r="F38" s="22" t="n"/>
+      <c r="G38" s="22" t="n"/>
+      <c r="H38" s="22" t="n"/>
+      <c r="I38" s="22" t="n"/>
+      <c r="J38" s="22" t="n"/>
+      <c r="K38" s="22" t="n"/>
+      <c r="L38" s="22" t="n"/>
+      <c r="M38" s="22" t="n"/>
+      <c r="N38" s="22" t="n"/>
+    </row>
+    <row r="39" ht="15.75" customHeight="1">
+      <c r="A39" s="22" t="n"/>
+      <c r="B39" s="22" t="n"/>
+      <c r="C39" s="22" t="n"/>
+      <c r="D39" s="22" t="n"/>
+      <c r="E39" s="22" t="n"/>
+      <c r="F39" s="22" t="n"/>
+      <c r="G39" s="22" t="n"/>
+      <c r="H39" s="22" t="n"/>
+      <c r="I39" s="22" t="n"/>
+      <c r="J39" s="22" t="n"/>
+      <c r="K39" s="22" t="n"/>
+      <c r="L39" s="22" t="n"/>
+      <c r="M39" s="22" t="n"/>
+      <c r="N39" s="22" t="n"/>
+    </row>
     <row r="40" ht="15.75" customHeight="1"/>
     <row r="41" ht="15.75" customHeight="1"/>
     <row r="42" ht="15.75" customHeight="1"/>
@@ -1757,170 +2756,210 @@
     <row r="998" ht="15.75" customHeight="1"/>
     <row r="999" ht="15.75" customHeight="1"/>
     <row r="1000" ht="15.75" customHeight="1"/>
-    <row r="1001" ht="15.75" customHeight="1"/>
-    <row r="1002" ht="15.75" customHeight="1"/>
-    <row r="1003" ht="15.75" customHeight="1"/>
-    <row r="1004" ht="15.75" customHeight="1"/>
-    <row r="1005" ht="15.75" customHeight="1"/>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <mergeCells count="5">
+    <mergeCell ref="D2:F2"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A16:E16"/>
+    <mergeCell ref="G2:J2"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
+  <pageSetup orientation="landscape"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1000"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="14.3984375" defaultRowHeight="15" customHeight="1"/>
+  <dimension ref="A1:B19"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="6.1328125" customWidth="1"/>
-    <col min="2" max="2" width="100" customWidth="1"/>
-    <col min="3" max="6" width="14.3984375" customWidth="1"/>
+    <col width="6.140625" customWidth="1" min="1" max="1"/>
+    <col width="100" customWidth="1" min="2" max="2"/>
+    <col width="14.42578125" customWidth="1" min="3" max="26"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="15.75" customHeight="1">
-      <c r="A1" s="5"/>
-    </row>
-    <row r="2" spans="1:2" ht="15.75" customHeight="1">
-      <c r="A2" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="B2" s="8" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="15.75" customHeight="1">
-      <c r="A3" s="9">
+    <row r="1" ht="15.75" customHeight="1">
+      <c r="A1" s="1" t="n"/>
+    </row>
+    <row r="2" ht="15.75" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>IMPACTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="15.75" customHeight="1">
+      <c r="A3" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="10" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="15.75" customHeight="1">
-      <c r="A4" s="9">
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>Despreciable: Poco relevante.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="15.75" customHeight="1">
+      <c r="A4" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="10" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="15.75" customHeight="1">
-      <c r="A5" s="9">
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>Marginal: Su impacto debe ser tenido en cuenta, pero no afecta factores claves del proyecto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="15.75" customHeight="1">
+      <c r="A5" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="B5" s="10" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="15.75" customHeight="1">
-      <c r="A6" s="9">
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Crítica: Podría afectar de manera sustancial al proyecto y podría impedir su conclusión/término de manera exitosa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="15.75" customHeight="1">
+      <c r="A6" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B6" s="10" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" ht="15.75" customHeight="1">
-      <c r="A7" s="6"/>
-    </row>
-    <row r="8" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="9" spans="1:2" ht="15.75" customHeight="1">
-      <c r="A9" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="B9" s="12" t="s">
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Catastrófica: Significaría el fracaso del proyecto o afectaría gravemente la ejecución/continuación/termino del mismo</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="15.75" customHeight="1">
+      <c r="A7" s="10" t="n"/>
+    </row>
+    <row r="8" ht="15.75" customHeight="1"/>
+    <row r="9" ht="15.75" customHeight="1">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>Probabilidad</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="15.75" customHeight="1">
+      <c r="A10" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="B10" s="14" t="inlineStr">
+        <is>
+          <t>Muy Bajo (Menos del 10%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="15.75" customHeight="1">
+      <c r="A11" s="13" t="n">
         <v>2</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" ht="15.75" customHeight="1">
-      <c r="A10" s="13">
+      <c r="B11" s="14" t="inlineStr">
+        <is>
+          <t>Bajo (Entre del 11% y 40%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="15.75" customHeight="1">
+      <c r="A12" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="B12" s="14" t="inlineStr">
+        <is>
+          <t>Medio (Entre  41 % y 80%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="15.75" customHeight="1">
+      <c r="A13" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="B13" s="14" t="inlineStr">
+        <is>
+          <t>Alto (Mas del 81%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="15.75" customHeight="1"/>
+    <row r="15" ht="15.75" customHeight="1">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>Categoria</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="15.75" customHeight="1">
+      <c r="A16" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="B10" s="14" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" ht="15.75" customHeight="1">
-      <c r="A11" s="13">
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t>Naturaleza</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="15.75" customHeight="1">
+      <c r="A17" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="B11" s="14" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" ht="15.75" customHeight="1">
-      <c r="A12" s="13">
+      <c r="B17" s="18" t="inlineStr">
+        <is>
+          <t>Externo</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="15.75" customHeight="1">
+      <c r="A18" s="17" t="n">
         <v>3</v>
       </c>
-      <c r="B12" s="14" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" ht="15.75" customHeight="1">
-      <c r="A13" s="13">
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>Desarrollo</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="15.75" customHeight="1">
+      <c r="A19" s="17" t="n">
         <v>4</v>
       </c>
-      <c r="B13" s="14" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="15" spans="1:2" ht="15.75" customHeight="1">
-      <c r="A15" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="B15" s="16" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" ht="15.75" customHeight="1">
-      <c r="A16" s="17">
-        <v>1</v>
-      </c>
-      <c r="B16" s="18" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" ht="15.75" customHeight="1">
-      <c r="A17" s="17">
-        <v>2</v>
-      </c>
-      <c r="B17" s="18" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" ht="15.75" customHeight="1">
-      <c r="A18" s="17">
-        <v>3</v>
-      </c>
-      <c r="B18" s="18" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" ht="15.75" customHeight="1">
-      <c r="A19" s="17">
-        <v>4</v>
-      </c>
-      <c r="B19" s="18" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="21" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="22" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="23" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="24" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="25" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="26" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="27" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="28" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="29" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="30" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="31" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="32" spans="1:2" ht="15.75" customHeight="1"/>
+      <c r="B19" s="18" t="inlineStr">
+        <is>
+          <t>Proyecto</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="15.75" customHeight="1"/>
+    <row r="21" ht="15.75" customHeight="1"/>
+    <row r="22" ht="15.75" customHeight="1"/>
+    <row r="23" ht="15.75" customHeight="1"/>
+    <row r="24" ht="15.75" customHeight="1"/>
+    <row r="25" ht="15.75" customHeight="1"/>
+    <row r="26" ht="15.75" customHeight="1"/>
+    <row r="27" ht="15.75" customHeight="1"/>
+    <row r="28" ht="15.75" customHeight="1"/>
+    <row r="29" ht="15.75" customHeight="1"/>
+    <row r="30" ht="15.75" customHeight="1"/>
+    <row r="31" ht="15.75" customHeight="1"/>
+    <row r="32" ht="15.75" customHeight="1"/>
     <row r="33" ht="15.75" customHeight="1"/>
     <row r="34" ht="15.75" customHeight="1"/>
     <row r="35" ht="15.75" customHeight="1"/>
@@ -2890,6 +3929,7 @@
     <row r="999" ht="15.75" customHeight="1"/>
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
+  <pageSetup orientation="landscape"/>
 </worksheet>
 </file>
</xml_diff>